<commit_message>
feat: FM-CT-5 impact survey DTI header, user manual link in nav, official form templates
- Add DTI FM-CT-5 official header to ImpactSurvey page (logo, doc code, version)
- Add User Manual link to PublicLayout, ParticipantLayout, OrganizerLayout headers
- Serve USER-MANUAL.html as static file at /docs/USER-MANUAL.html
- Update impact survey email template to reference FM-CT-5
- Update User Manual Section 10 with detailed FM-CT-5 form description
- Add OrganizerAttendanceSheet (FM-CT-2A) print-ready A4 landscape
- Add OrganizerChecklistPrint (FM-CT-7) print-ready A4 portrait
- Add DTI logo to CsfSurvey and OrganizerCsfReport headers
- Add attendance-sheet backend endpoint with enriched demographics
- Add MySurveyResponses viewer, OrganizerProposalList page
- Various UI fixes: certificate PDF download, CSF deduplication, admin users
</commit_message>
<xml_diff>
--- a/docs/5. Pilot Collaboration with Cubeworks/FM-CT-2Av1_External Attendance Sheet.xlsx
+++ b/docs/5. Pilot Collaboration with Cubeworks/FM-CT-2Av1_External Attendance Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timmyjoylomarda\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cubeworks/Documents/DTI Region 7/EMS Dash/docs/5. Pilot Collaboration with Cubeworks/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D26C27-E842-4FB1-ADA2-D7A8489318E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -1115,23 +1115,41 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1181,29 +1199,11 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1623,197 +1623,196 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:W52"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="16.8" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.109375" style="16" customWidth="1"/>
+    <col min="1" max="1" width="3.1640625" style="16" customWidth="1"/>
     <col min="2" max="2" width="40.6640625" style="13" customWidth="1"/>
     <col min="3" max="3" width="4.6640625" style="13" customWidth="1"/>
-    <col min="4" max="4" width="5.109375" style="12" customWidth="1"/>
+    <col min="4" max="4" width="5.1640625" style="12" customWidth="1"/>
     <col min="5" max="5" width="7.6640625" style="12" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" style="12" customWidth="1"/>
     <col min="7" max="7" width="7" style="12" customWidth="1"/>
-    <col min="8" max="8" width="8.5546875" style="18" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" style="18" customWidth="1"/>
-    <col min="10" max="10" width="8.5546875" style="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.44140625" style="18" customWidth="1"/>
-    <col min="12" max="12" width="7.109375" style="18" customWidth="1"/>
-    <col min="13" max="13" width="5.88671875" style="18" customWidth="1"/>
+    <col min="8" max="8" width="8.5" style="18" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" style="18" customWidth="1"/>
+    <col min="10" max="10" width="8.5" style="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5" style="18" customWidth="1"/>
+    <col min="12" max="12" width="7.1640625" style="18" customWidth="1"/>
+    <col min="13" max="13" width="5.83203125" style="18" customWidth="1"/>
     <col min="14" max="14" width="7.6640625" style="18" customWidth="1"/>
     <col min="15" max="15" width="8.6640625" style="18" customWidth="1"/>
-    <col min="16" max="16" width="8.109375" style="18" customWidth="1"/>
-    <col min="17" max="17" width="6.44140625" style="18" customWidth="1"/>
-    <col min="18" max="18" width="7.44140625" style="18" customWidth="1"/>
-    <col min="19" max="19" width="18.5546875" style="12" customWidth="1"/>
-    <col min="20" max="20" width="18.44140625" style="12" customWidth="1"/>
+    <col min="16" max="16" width="8.1640625" style="18" customWidth="1"/>
+    <col min="17" max="17" width="6.5" style="18" customWidth="1"/>
+    <col min="18" max="18" width="7.5" style="18" customWidth="1"/>
+    <col min="19" max="20" width="18.5" style="12" customWidth="1"/>
     <col min="21" max="21" width="18.6640625" style="15" customWidth="1"/>
     <col min="22" max="22" width="13.6640625" style="14" customWidth="1"/>
     <col min="23" max="23" width="18" style="4" customWidth="1"/>
-    <col min="24" max="16384" width="9.109375" style="4"/>
+    <col min="24" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:23" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="1:23" ht="88.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="111" t="s">
+    <row r="2" spans="1:23" ht="18" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:23" ht="88.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="117" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="112"/>
+      <c r="B3" s="118"/>
       <c r="C3" s="78"/>
-      <c r="D3" s="125" t="s">
+      <c r="D3" s="131" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="126"/>
-      <c r="Q3" s="126"/>
-      <c r="R3" s="126"/>
-      <c r="S3" s="126"/>
-      <c r="T3" s="126"/>
-      <c r="U3" s="122" t="s">
+      <c r="E3" s="132"/>
+      <c r="F3" s="132"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="132"/>
+      <c r="I3" s="132"/>
+      <c r="J3" s="132"/>
+      <c r="K3" s="132"/>
+      <c r="L3" s="132"/>
+      <c r="M3" s="132"/>
+      <c r="N3" s="132"/>
+      <c r="O3" s="132"/>
+      <c r="P3" s="132"/>
+      <c r="Q3" s="132"/>
+      <c r="R3" s="132"/>
+      <c r="S3" s="132"/>
+      <c r="T3" s="132"/>
+      <c r="U3" s="128" t="s">
         <v>32</v>
       </c>
-      <c r="V3" s="123"/>
-      <c r="W3" s="124"/>
-    </row>
-    <row r="4" spans="1:23" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="113" t="s">
+      <c r="V3" s="129"/>
+      <c r="W3" s="130"/>
+    </row>
+    <row r="4" spans="1:23" s="5" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="119" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="114"/>
-      <c r="C4" s="114"/>
-      <c r="D4" s="114"/>
-      <c r="E4" s="114"/>
-      <c r="F4" s="114"/>
-      <c r="G4" s="114"/>
-      <c r="H4" s="114"/>
-      <c r="I4" s="114"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="114"/>
-      <c r="L4" s="114"/>
-      <c r="M4" s="114"/>
-      <c r="N4" s="114"/>
-      <c r="O4" s="114"/>
-      <c r="P4" s="114"/>
-      <c r="Q4" s="114"/>
-      <c r="R4" s="114"/>
-      <c r="S4" s="114"/>
-      <c r="T4" s="114"/>
-      <c r="U4" s="114"/>
-      <c r="V4" s="116" t="s">
+      <c r="B4" s="120"/>
+      <c r="C4" s="120"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="120"/>
+      <c r="G4" s="120"/>
+      <c r="H4" s="120"/>
+      <c r="I4" s="120"/>
+      <c r="J4" s="120"/>
+      <c r="K4" s="120"/>
+      <c r="L4" s="120"/>
+      <c r="M4" s="120"/>
+      <c r="N4" s="120"/>
+      <c r="O4" s="120"/>
+      <c r="P4" s="120"/>
+      <c r="Q4" s="120"/>
+      <c r="R4" s="120"/>
+      <c r="S4" s="120"/>
+      <c r="T4" s="120"/>
+      <c r="U4" s="120"/>
+      <c r="V4" s="122" t="s">
         <v>3</v>
       </c>
-      <c r="W4" s="117"/>
-    </row>
-    <row r="5" spans="1:23" s="6" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="113"/>
-      <c r="B5" s="114"/>
-      <c r="C5" s="114"/>
-      <c r="D5" s="114"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="114"/>
-      <c r="K5" s="114"/>
-      <c r="L5" s="114"/>
-      <c r="M5" s="114"/>
-      <c r="N5" s="114"/>
-      <c r="O5" s="114"/>
-      <c r="P5" s="114"/>
-      <c r="Q5" s="114"/>
-      <c r="R5" s="114"/>
-      <c r="S5" s="114"/>
-      <c r="T5" s="114"/>
-      <c r="U5" s="114"/>
-      <c r="V5" s="118" t="s">
+      <c r="W4" s="123"/>
+    </row>
+    <row r="5" spans="1:23" s="6" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="119"/>
+      <c r="B5" s="120"/>
+      <c r="C5" s="120"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="120"/>
+      <c r="H5" s="120"/>
+      <c r="I5" s="120"/>
+      <c r="J5" s="120"/>
+      <c r="K5" s="120"/>
+      <c r="L5" s="120"/>
+      <c r="M5" s="120"/>
+      <c r="N5" s="120"/>
+      <c r="O5" s="120"/>
+      <c r="P5" s="120"/>
+      <c r="Q5" s="120"/>
+      <c r="R5" s="120"/>
+      <c r="S5" s="120"/>
+      <c r="T5" s="120"/>
+      <c r="U5" s="120"/>
+      <c r="V5" s="124" t="s">
         <v>4</v>
       </c>
-      <c r="W5" s="119"/>
-    </row>
-    <row r="6" spans="1:23" s="7" customFormat="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="113"/>
-      <c r="B6" s="114"/>
-      <c r="C6" s="115"/>
-      <c r="D6" s="115"/>
-      <c r="E6" s="115"/>
-      <c r="F6" s="115"/>
-      <c r="G6" s="115"/>
-      <c r="H6" s="115"/>
-      <c r="I6" s="115"/>
-      <c r="J6" s="115"/>
-      <c r="K6" s="115"/>
-      <c r="L6" s="115"/>
-      <c r="M6" s="115"/>
-      <c r="N6" s="115"/>
-      <c r="O6" s="115"/>
-      <c r="P6" s="115"/>
-      <c r="Q6" s="115"/>
-      <c r="R6" s="115"/>
-      <c r="S6" s="115"/>
-      <c r="T6" s="115"/>
-      <c r="U6" s="115"/>
-      <c r="V6" s="120" t="s">
+      <c r="W5" s="125"/>
+    </row>
+    <row r="6" spans="1:23" s="7" customFormat="1" ht="18" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="119"/>
+      <c r="B6" s="120"/>
+      <c r="C6" s="121"/>
+      <c r="D6" s="121"/>
+      <c r="E6" s="121"/>
+      <c r="F6" s="121"/>
+      <c r="G6" s="121"/>
+      <c r="H6" s="121"/>
+      <c r="I6" s="121"/>
+      <c r="J6" s="121"/>
+      <c r="K6" s="121"/>
+      <c r="L6" s="121"/>
+      <c r="M6" s="121"/>
+      <c r="N6" s="121"/>
+      <c r="O6" s="121"/>
+      <c r="P6" s="121"/>
+      <c r="Q6" s="121"/>
+      <c r="R6" s="121"/>
+      <c r="S6" s="121"/>
+      <c r="T6" s="121"/>
+      <c r="U6" s="121"/>
+      <c r="V6" s="126" t="s">
         <v>5</v>
       </c>
-      <c r="W6" s="121"/>
-    </row>
-    <row r="7" spans="1:23" s="8" customFormat="1" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="127" t="s">
+      <c r="W6" s="127"/>
+    </row>
+    <row r="7" spans="1:23" s="8" customFormat="1" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="105" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="128"/>
+      <c r="B7" s="106"/>
       <c r="C7" s="109" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="110"/>
+      <c r="D7" s="111"/>
       <c r="E7" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="131"/>
-      <c r="G7" s="110"/>
-      <c r="H7" s="132" t="s">
+      <c r="F7" s="110"/>
+      <c r="G7" s="111"/>
+      <c r="H7" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="132"/>
-      <c r="J7" s="133"/>
-      <c r="K7" s="134" t="s">
+      <c r="I7" s="112"/>
+      <c r="J7" s="113"/>
+      <c r="K7" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="L7" s="132"/>
-      <c r="M7" s="132"/>
-      <c r="N7" s="132"/>
-      <c r="O7" s="132"/>
-      <c r="P7" s="132"/>
-      <c r="Q7" s="132"/>
-      <c r="R7" s="133"/>
-      <c r="S7" s="107" t="s">
+      <c r="L7" s="112"/>
+      <c r="M7" s="112"/>
+      <c r="N7" s="112"/>
+      <c r="O7" s="112"/>
+      <c r="P7" s="112"/>
+      <c r="Q7" s="112"/>
+      <c r="R7" s="113"/>
+      <c r="S7" s="115" t="s">
         <v>11</v>
       </c>
-      <c r="T7" s="107" t="s">
+      <c r="T7" s="115" t="s">
         <v>12</v>
       </c>
-      <c r="U7" s="107" t="s">
+      <c r="U7" s="115" t="s">
         <v>13</v>
       </c>
-      <c r="V7" s="107" t="s">
+      <c r="V7" s="115" t="s">
         <v>14</v>
       </c>
-      <c r="W7" s="105" t="s">
+      <c r="W7" s="133" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:23" s="10" customFormat="1" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="129"/>
-      <c r="B8" s="130"/>
+    <row r="8" spans="1:23" s="10" customFormat="1" ht="56.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="107"/>
+      <c r="B8" s="108"/>
       <c r="C8" s="79" t="s">
         <v>16</v>
       </c>
@@ -1862,13 +1861,13 @@
       <c r="R8" s="83" t="s">
         <v>31</v>
       </c>
-      <c r="S8" s="108"/>
-      <c r="T8" s="108"/>
-      <c r="U8" s="108"/>
-      <c r="V8" s="108"/>
-      <c r="W8" s="106"/>
-    </row>
-    <row r="9" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="S8" s="116"/>
+      <c r="T8" s="116"/>
+      <c r="U8" s="116"/>
+      <c r="V8" s="116"/>
+      <c r="W8" s="134"/>
+    </row>
+    <row r="9" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="84">
         <v>1</v>
       </c>
@@ -1895,7 +1894,7 @@
       <c r="V9" s="95"/>
       <c r="W9" s="95"/>
     </row>
-    <row r="10" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="84">
         <v>2</v>
       </c>
@@ -1922,7 +1921,7 @@
       <c r="V10" s="104"/>
       <c r="W10" s="104"/>
     </row>
-    <row r="11" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="51">
         <v>3</v>
       </c>
@@ -1949,7 +1948,7 @@
       <c r="V11" s="45"/>
       <c r="W11" s="45"/>
     </row>
-    <row r="12" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="51">
         <v>4</v>
       </c>
@@ -1976,7 +1975,7 @@
       <c r="V12" s="45"/>
       <c r="W12" s="45"/>
     </row>
-    <row r="13" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="51">
         <v>5</v>
       </c>
@@ -2003,7 +2002,7 @@
       <c r="V13" s="45"/>
       <c r="W13" s="45"/>
     </row>
-    <row r="14" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="51">
         <v>6</v>
       </c>
@@ -2030,7 +2029,7 @@
       <c r="V14" s="45"/>
       <c r="W14" s="45"/>
     </row>
-    <row r="15" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="51">
         <v>7</v>
       </c>
@@ -2057,7 +2056,7 @@
       <c r="V15" s="45"/>
       <c r="W15" s="45"/>
     </row>
-    <row r="16" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="51">
         <v>8</v>
       </c>
@@ -2084,7 +2083,7 @@
       <c r="V16" s="45"/>
       <c r="W16" s="45"/>
     </row>
-    <row r="17" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="51">
         <v>9</v>
       </c>
@@ -2111,7 +2110,7 @@
       <c r="V17" s="45"/>
       <c r="W17" s="45"/>
     </row>
-    <row r="18" spans="1:23" s="11" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" s="11" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="51">
         <v>10</v>
       </c>
@@ -2138,7 +2137,7 @@
       <c r="V18" s="46"/>
       <c r="W18" s="48"/>
     </row>
-    <row r="19" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="51">
         <v>11</v>
       </c>
@@ -2165,7 +2164,7 @@
       <c r="V19" s="46"/>
       <c r="W19" s="48"/>
     </row>
-    <row r="20" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="51">
         <v>12</v>
       </c>
@@ -2192,7 +2191,7 @@
       <c r="V20" s="46"/>
       <c r="W20" s="48"/>
     </row>
-    <row r="21" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="51">
         <v>13</v>
       </c>
@@ -2219,7 +2218,7 @@
       <c r="V21" s="62"/>
       <c r="W21" s="63"/>
     </row>
-    <row r="22" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="51">
         <v>14</v>
       </c>
@@ -2246,7 +2245,7 @@
       <c r="V22" s="62"/>
       <c r="W22" s="63"/>
     </row>
-    <row r="23" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="51">
         <v>15</v>
       </c>
@@ -2273,7 +2272,7 @@
       <c r="V23" s="47"/>
       <c r="W23" s="49"/>
     </row>
-    <row r="24" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9"/>
       <c r="B24" s="64"/>
       <c r="C24" s="64"/>
@@ -2298,7 +2297,7 @@
       <c r="V24" s="68"/>
       <c r="W24" s="69"/>
     </row>
-    <row r="25" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
       <c r="B25" s="64"/>
       <c r="C25" s="64"/>
@@ -2323,7 +2322,7 @@
       <c r="V25" s="68"/>
       <c r="W25" s="70"/>
     </row>
-    <row r="26" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>16</v>
       </c>
@@ -2350,7 +2349,7 @@
       <c r="V26" s="68"/>
       <c r="W26" s="70"/>
     </row>
-    <row r="27" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>17</v>
       </c>
@@ -2377,7 +2376,7 @@
       <c r="V27" s="68"/>
       <c r="W27" s="69"/>
     </row>
-    <row r="28" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>18</v>
       </c>
@@ -2404,7 +2403,7 @@
       <c r="V28" s="72"/>
       <c r="W28" s="70"/>
     </row>
-    <row r="29" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" s="10" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>19</v>
       </c>
@@ -2431,7 +2430,7 @@
       <c r="V29" s="68"/>
       <c r="W29" s="70"/>
     </row>
-    <row r="31" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>20</v>
       </c>
@@ -2441,7 +2440,7 @@
       <c r="V31" s="75"/>
       <c r="W31" s="5"/>
     </row>
-    <row r="32" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
         <v>21</v>
       </c>
@@ -2449,7 +2448,7 @@
       <c r="V32" s="75"/>
       <c r="W32" s="5"/>
     </row>
-    <row r="33" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
         <v>22</v>
       </c>
@@ -2459,7 +2458,7 @@
       <c r="V33" s="75"/>
       <c r="W33" s="5"/>
     </row>
-    <row r="34" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
         <v>23</v>
       </c>
@@ -2469,7 +2468,7 @@
       <c r="V34" s="75"/>
       <c r="W34" s="5"/>
     </row>
-    <row r="35" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
         <v>24</v>
       </c>
@@ -2479,7 +2478,7 @@
       <c r="V35" s="75"/>
       <c r="W35" s="5"/>
     </row>
-    <row r="36" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
         <v>25</v>
       </c>
@@ -2489,7 +2488,7 @@
       <c r="V36" s="75"/>
       <c r="W36" s="5"/>
     </row>
-    <row r="37" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
         <v>26</v>
       </c>
@@ -2499,7 +2498,7 @@
       <c r="V37" s="75"/>
       <c r="W37" s="5"/>
     </row>
-    <row r="38" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
         <v>27</v>
       </c>
@@ -2509,7 +2508,7 @@
       <c r="V38" s="75"/>
       <c r="W38" s="5"/>
     </row>
-    <row r="39" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
         <v>28</v>
       </c>
@@ -2519,7 +2518,7 @@
       <c r="V39" s="75"/>
       <c r="W39" s="5"/>
     </row>
-    <row r="40" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
         <v>29</v>
       </c>
@@ -2529,7 +2528,7 @@
       <c r="V40" s="75"/>
       <c r="W40" s="5"/>
     </row>
-    <row r="41" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
         <v>30</v>
       </c>
@@ -2539,7 +2538,7 @@
       <c r="V41" s="75"/>
       <c r="W41" s="5"/>
     </row>
-    <row r="42" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
         <v>31</v>
       </c>
@@ -2547,7 +2546,7 @@
       <c r="C42" s="64"/>
       <c r="U42" s="13"/>
     </row>
-    <row r="43" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
         <v>32</v>
       </c>
@@ -2555,55 +2554,55 @@
       <c r="C43" s="64"/>
       <c r="U43" s="13"/>
     </row>
-    <row r="44" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="9"/>
       <c r="B44" s="64"/>
       <c r="C44" s="64"/>
       <c r="U44" s="13"/>
     </row>
-    <row r="45" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="9"/>
       <c r="B45" s="77"/>
       <c r="C45" s="77"/>
     </row>
-    <row r="46" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
         <v>33</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="9">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="9">
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="9"/>
     </row>
-    <row r="50" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="9"/>
       <c r="B50" s="77"/>
       <c r="C50" s="77"/>
     </row>
-    <row r="51" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="9">
         <v>36</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A7:B8"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="K7:R7"/>
-    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="W7:W8"/>
+    <mergeCell ref="S7:S8"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="V7:V8"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:U6"/>
     <mergeCell ref="V4:W4"/>
@@ -2611,13 +2610,13 @@
     <mergeCell ref="V6:W6"/>
     <mergeCell ref="U3:W3"/>
     <mergeCell ref="D3:T3"/>
-    <mergeCell ref="W7:W8"/>
-    <mergeCell ref="S7:S8"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="V7:V8"/>
+    <mergeCell ref="A7:B8"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="K7:R7"/>
+    <mergeCell ref="U7:U8"/>
   </mergeCells>
-  <conditionalFormatting sqref="S61:T68 S9:T28 D27:R28 D10:R24 D8:R8 D61:R76 D50:R57">
+  <conditionalFormatting sqref="D8:R8 S9:T28 D10:R24 D27:R28 D50:R57 S61:T68 D61:R76">
     <cfRule type="containsText" dxfId="2" priority="10" operator="containsText" text="pacheco">
       <formula>NOT(ISERROR(SEARCH("pacheco",D8)))</formula>
     </cfRule>
@@ -2636,21 +2635,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B1746A42879D3440A6E46657556E1CED" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d7328c36335228196cf86f090fcb920">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bd93ad54-4974-4828-a527-cd17d078195f" xmlns:ns3="2f74224c-65ea-495e-8d51-9349cddd824e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9bdb2fb4b22f0836efd288cee492c383" ns2:_="" ns3:_="">
     <xsd:import namespace="bd93ad54-4974-4828-a527-cd17d078195f"/>
@@ -2879,10 +2863,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83A600FA-C94E-47A9-B4F0-6F22BB6B39F1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B0A5066-76ED-40E1-ABF4-41259FBA11D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bd93ad54-4974-4828-a527-cd17d078195f"/>
+    <ds:schemaRef ds:uri="2f74224c-65ea-495e-8d51-9349cddd824e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2905,5 +2915,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B0A5066-76ED-40E1-ABF4-41259FBA11D9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83A600FA-C94E-47A9-B4F0-6F22BB6B39F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>